<commit_message>
Make Content List items separate Content Items
The Content List becomes a container: More stays a property of the
list and each referenced page is its own Content Item, so authors can
add, reorder and remove items in the Universal Editor. The first four
items are shown (later ones appear dimmed while editing); lists in the
previous format still render. The homepage importer writes the new
structure. Links to AEM paths (/content/...) are no longer rewritten
to the source site on import.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-full.report.xlsx
+++ b/tools/importer/reports/import-article-full.report.xlsx
@@ -67,7 +67,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-29T03:18:55.011Z</t>
+    <t>2026-09-29T04:46:35.577Z</t>
   </si>
   <si>
     <t>EMA: Department of Conservation</t>
@@ -94,7 +94,7 @@
     <t>article-hero</t>
   </si>
   <si>
-    <t>2026-09-29T03:19:03.033Z</t>
+    <t>2026-09-29T04:46:45.639Z</t>
   </si>
   <si>
     <t>EMA: Bird flu updates: Issues</t>
@@ -115,7 +115,7 @@
     <t>The Conservation Amendment Bill aims to modernise the way conservation land is managed, support economic growth, and deliver stronger conservation outcomes.</t>
   </si>
   <si>
-    <t>2026-09-29T03:19:16.392Z</t>
+    <t>2026-09-29T04:47:00.105Z</t>
   </si>
   <si>
     <t>EMA: Conservation Amendment Bill: Managing conservation</t>
@@ -142,7 +142,7 @@
     <t>article-full</t>
   </si>
   <si>
-    <t>2026-09-29T03:51:05.157Z</t>
+    <t>2026-09-29T04:48:31.038Z</t>
   </si>
   <si>
     <t>EMA: National Wild Goat Hunting Competition 2026</t>
@@ -166,7 +166,7 @@
     <t>A four-wheel drive (4WD) club has joined forces with the Department of Conservation to fund and plant native shrubs and trees to help cover damage done by vehicles.</t>
   </si>
   <si>
-    <t>2026-09-29T03:19:42.140Z</t>
+    <t>2026-09-29T04:47:18.316Z</t>
   </si>
   <si>
     <t>EMA: 4WD group plants native trees to fix damage</t>
@@ -184,7 +184,7 @@
     <t>The government is boosting support for wildlife care facilities because of their key role in New Zealand’s bird flu surveillance and response, Conservation Minister Tama Potaka and Biosecurity Minister Andrew Hoggard say.</t>
   </si>
   <si>
-    <t>2026-09-29T03:19:30.980Z</t>
+    <t>2026-09-29T04:47:06.080Z</t>
   </si>
   <si>
     <t>EMA: Funding boost for bird flu surveillance: Media release 24 September 2026</t>
@@ -205,7 +205,7 @@
     <t>The Government is taking a practical step to address contaminated sites on Crown-owned land.</t>
   </si>
   <si>
-    <t>2026-09-29T03:19:36.448Z</t>
+    <t>2026-09-29T04:47:12.522Z</t>
   </si>
   <si>
     <t>EMA: Government invests in cleaning up contaminated Crown land: Media release 23 September 2026</t>
@@ -226,7 +226,7 @@
     <t>DOC has confirmed toxoplasmosis was the cause of death of a pregnant Hector’s dolphin found at Invercargill’s Oreti Beach last month.</t>
   </si>
   <si>
-    <t>2026-09-29T03:19:49.230Z</t>
+    <t>2026-09-29T04:47:24.688Z</t>
   </si>
   <si>
     <t>EMA: Toxoplasmosis confirmed as cause of death of pregnant Hector’s dolphin: Media release 22 September 2026</t>
@@ -247,7 +247,7 @@
     <t>The whitebait fishing season is open. Find out when, where and how to fish for whitebait in New Zealand and the Chatham Islands.</t>
   </si>
   <si>
-    <t>2026-09-29T03:19:09.164Z</t>
+    <t>2026-09-29T04:46:54.364Z</t>
   </si>
   <si>
     <t>EMA: Whitebaiting: Things to do</t>
@@ -271,7 +271,7 @@
     <t>Discover some of our best short walks. They’re easy to get to and great for families – there’s something for everyone.</t>
   </si>
   <si>
-    <t>2026-09-29T03:20:14.137Z</t>
+    <t>2026-09-29T04:48:19.394Z</t>
   </si>
   <si>
     <t>EMA: Short Walks: Walking and tramping</t>

</xml_diff>

<commit_message>
Add hero image info bubble and alt text
The hero gets an Alt text field on its image and optional Image caption
and Image credit fields, shown in an info bubble opened from a button
at the top right of the image, as on the source. The importer reads
each page's caption and credit from the source page's own HTML (the
live page only renders them on click) through a new onLoad step.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-full.report.xlsx
+++ b/tools/importer/reports/import-article-full.report.xlsx
@@ -67,7 +67,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-29T04:46:35.577Z</t>
+    <t>2026-09-29T05:48:27.130Z</t>
   </si>
   <si>
     <t>EMA: Department of Conservation</t>
@@ -94,7 +94,7 @@
     <t>article-hero</t>
   </si>
   <si>
-    <t>2026-09-29T04:46:45.639Z</t>
+    <t>2026-09-29T05:48:36.788Z</t>
   </si>
   <si>
     <t>EMA: Bird flu updates: Issues</t>
@@ -115,7 +115,7 @@
     <t>The Conservation Amendment Bill aims to modernise the way conservation land is managed, support economic growth, and deliver stronger conservation outcomes.</t>
   </si>
   <si>
-    <t>2026-09-29T04:47:00.105Z</t>
+    <t>2026-09-29T05:48:49.691Z</t>
   </si>
   <si>
     <t>EMA: Conservation Amendment Bill: Managing conservation</t>
@@ -142,7 +142,7 @@
     <t>article-full</t>
   </si>
   <si>
-    <t>2026-09-29T04:48:31.038Z</t>
+    <t>2026-09-29T05:50:12.484Z</t>
   </si>
   <si>
     <t>EMA: National Wild Goat Hunting Competition 2026</t>
@@ -166,7 +166,7 @@
     <t>A four-wheel drive (4WD) club has joined forces with the Department of Conservation to fund and plant native shrubs and trees to help cover damage done by vehicles.</t>
   </si>
   <si>
-    <t>2026-09-29T04:47:18.316Z</t>
+    <t>2026-09-29T05:49:08.031Z</t>
   </si>
   <si>
     <t>EMA: 4WD group plants native trees to fix damage</t>
@@ -184,7 +184,7 @@
     <t>The government is boosting support for wildlife care facilities because of their key role in New Zealand’s bird flu surveillance and response, Conservation Minister Tama Potaka and Biosecurity Minister Andrew Hoggard say.</t>
   </si>
   <si>
-    <t>2026-09-29T04:47:06.080Z</t>
+    <t>2026-09-29T05:48:56.720Z</t>
   </si>
   <si>
     <t>EMA: Funding boost for bird flu surveillance: Media release 24 September 2026</t>
@@ -205,7 +205,7 @@
     <t>The Government is taking a practical step to address contaminated sites on Crown-owned land.</t>
   </si>
   <si>
-    <t>2026-09-29T04:47:12.522Z</t>
+    <t>2026-09-29T05:49:02.558Z</t>
   </si>
   <si>
     <t>EMA: Government invests in cleaning up contaminated Crown land: Media release 23 September 2026</t>
@@ -226,7 +226,7 @@
     <t>DOC has confirmed toxoplasmosis was the cause of death of a pregnant Hector’s dolphin found at Invercargill’s Oreti Beach last month.</t>
   </si>
   <si>
-    <t>2026-09-29T04:47:24.688Z</t>
+    <t>2026-09-29T05:49:15.737Z</t>
   </si>
   <si>
     <t>EMA: Toxoplasmosis confirmed as cause of death of pregnant Hector’s dolphin: Media release 22 September 2026</t>
@@ -247,7 +247,7 @@
     <t>The whitebait fishing season is open. Find out when, where and how to fish for whitebait in New Zealand and the Chatham Islands.</t>
   </si>
   <si>
-    <t>2026-09-29T04:46:54.364Z</t>
+    <t>2026-09-29T05:48:42.473Z</t>
   </si>
   <si>
     <t>EMA: Whitebaiting: Things to do</t>
@@ -271,7 +271,7 @@
     <t>Discover some of our best short walks. They’re easy to get to and great for families – there’s something for everyone.</t>
   </si>
   <si>
-    <t>2026-09-29T04:48:19.394Z</t>
+    <t>2026-09-29T05:50:00.592Z</t>
   </si>
   <si>
     <t>EMA: Short Walks: Walking and tramping</t>

</xml_diff>

<commit_message>
Read hero image info from the DAM asset metadata
The hero's caption fields are replaced by one Image info field
referencing the image's DAM asset. The info bubble reads the asset's
dc:title and dc:rights from AEM (Publish on the site, author while
editing) and shows "Image: <rights> | DOC" with the static copyright
link. The importer sets Image info to each hero's DAM image; the
source-caption onLoad step is removed.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-full.report.xlsx
+++ b/tools/importer/reports/import-article-full.report.xlsx
@@ -67,7 +67,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-29T05:48:27.130Z</t>
+    <t>2026-09-29T06:18:51.603Z</t>
   </si>
   <si>
     <t>EMA: Department of Conservation</t>
@@ -94,7 +94,7 @@
     <t>article-hero</t>
   </si>
   <si>
-    <t>2026-09-29T05:48:36.788Z</t>
+    <t>2026-09-29T06:19:01.849Z</t>
   </si>
   <si>
     <t>EMA: Bird flu updates: Issues</t>
@@ -115,7 +115,7 @@
     <t>The Conservation Amendment Bill aims to modernise the way conservation land is managed, support economic growth, and deliver stronger conservation outcomes.</t>
   </si>
   <si>
-    <t>2026-09-29T05:48:49.691Z</t>
+    <t>2026-09-29T06:19:15.244Z</t>
   </si>
   <si>
     <t>EMA: Conservation Amendment Bill: Managing conservation</t>
@@ -142,7 +142,7 @@
     <t>article-full</t>
   </si>
   <si>
-    <t>2026-09-29T05:50:12.484Z</t>
+    <t>2026-09-29T06:20:38.591Z</t>
   </si>
   <si>
     <t>EMA: National Wild Goat Hunting Competition 2026</t>
@@ -166,7 +166,7 @@
     <t>A four-wheel drive (4WD) club has joined forces with the Department of Conservation to fund and plant native shrubs and trees to help cover damage done by vehicles.</t>
   </si>
   <si>
-    <t>2026-09-29T05:49:08.031Z</t>
+    <t>2026-09-29T06:19:34.740Z</t>
   </si>
   <si>
     <t>EMA: 4WD group plants native trees to fix damage</t>
@@ -184,7 +184,7 @@
     <t>The government is boosting support for wildlife care facilities because of their key role in New Zealand’s bird flu surveillance and response, Conservation Minister Tama Potaka and Biosecurity Minister Andrew Hoggard say.</t>
   </si>
   <si>
-    <t>2026-09-29T05:48:56.720Z</t>
+    <t>2026-09-29T06:19:22.039Z</t>
   </si>
   <si>
     <t>EMA: Funding boost for bird flu surveillance: Media release 24 September 2026</t>
@@ -205,7 +205,7 @@
     <t>The Government is taking a practical step to address contaminated sites on Crown-owned land.</t>
   </si>
   <si>
-    <t>2026-09-29T05:49:02.558Z</t>
+    <t>2026-09-29T06:19:28.613Z</t>
   </si>
   <si>
     <t>EMA: Government invests in cleaning up contaminated Crown land: Media release 23 September 2026</t>
@@ -226,7 +226,7 @@
     <t>DOC has confirmed toxoplasmosis was the cause of death of a pregnant Hector’s dolphin found at Invercargill’s Oreti Beach last month.</t>
   </si>
   <si>
-    <t>2026-09-29T05:49:15.737Z</t>
+    <t>2026-09-29T06:19:42.918Z</t>
   </si>
   <si>
     <t>EMA: Toxoplasmosis confirmed as cause of death of pregnant Hector’s dolphin: Media release 22 September 2026</t>
@@ -247,7 +247,7 @@
     <t>The whitebait fishing season is open. Find out when, where and how to fish for whitebait in New Zealand and the Chatham Islands.</t>
   </si>
   <si>
-    <t>2026-09-29T05:48:42.473Z</t>
+    <t>2026-09-29T06:19:09.443Z</t>
   </si>
   <si>
     <t>EMA: Whitebaiting: Things to do</t>
@@ -271,7 +271,7 @@
     <t>Discover some of our best short walks. They’re easy to get to and great for families – there’s something for everyone.</t>
   </si>
   <si>
-    <t>2026-09-29T05:50:00.592Z</t>
+    <t>2026-09-29T06:20:27.992Z</t>
   </si>
   <si>
     <t>EMA: Short Walks: Walking and tramping</t>

</xml_diff>

<commit_message>
Read hero image info from the image file's XMP
AEM publishes a DAM image reference as an image, so the Image info
field never carried the asset path. The hero now reads dc:title and
dc:rights from the XMP embedded in the hero image itself (a partial
download of the original file, the same values AEM Assets extracts),
and the Image info field and its import row are removed.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-full.report.xlsx
+++ b/tools/importer/reports/import-article-full.report.xlsx
@@ -67,7 +67,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-29T06:18:51.603Z</t>
+    <t>2026-09-29T06:45:35.294Z</t>
   </si>
   <si>
     <t>EMA: Department of Conservation</t>
@@ -94,7 +94,7 @@
     <t>article-hero</t>
   </si>
   <si>
-    <t>2026-09-29T06:19:01.849Z</t>
+    <t>2026-09-29T06:45:44.683Z</t>
   </si>
   <si>
     <t>EMA: Bird flu updates: Issues</t>
@@ -115,7 +115,7 @@
     <t>The Conservation Amendment Bill aims to modernise the way conservation land is managed, support economic growth, and deliver stronger conservation outcomes.</t>
   </si>
   <si>
-    <t>2026-09-29T06:19:15.244Z</t>
+    <t>2026-09-29T06:45:57.265Z</t>
   </si>
   <si>
     <t>EMA: Conservation Amendment Bill: Managing conservation</t>
@@ -142,7 +142,7 @@
     <t>article-full</t>
   </si>
   <si>
-    <t>2026-09-29T06:20:38.591Z</t>
+    <t>2026-09-29T06:46:56.757Z</t>
   </si>
   <si>
     <t>EMA: National Wild Goat Hunting Competition 2026</t>
@@ -166,7 +166,7 @@
     <t>A four-wheel drive (4WD) club has joined forces with the Department of Conservation to fund and plant native shrubs and trees to help cover damage done by vehicles.</t>
   </si>
   <si>
-    <t>2026-09-29T06:19:34.740Z</t>
+    <t>2026-09-29T06:46:18.512Z</t>
   </si>
   <si>
     <t>EMA: 4WD group plants native trees to fix damage</t>
@@ -184,7 +184,7 @@
     <t>The government is boosting support for wildlife care facilities because of their key role in New Zealand’s bird flu surveillance and response, Conservation Minister Tama Potaka and Biosecurity Minister Andrew Hoggard say.</t>
   </si>
   <si>
-    <t>2026-09-29T06:19:22.039Z</t>
+    <t>2026-09-29T06:46:04.445Z</t>
   </si>
   <si>
     <t>EMA: Funding boost for bird flu surveillance: Media release 24 September 2026</t>
@@ -205,7 +205,7 @@
     <t>The Government is taking a practical step to address contaminated sites on Crown-owned land.</t>
   </si>
   <si>
-    <t>2026-09-29T06:19:28.613Z</t>
+    <t>2026-09-29T06:46:11.347Z</t>
   </si>
   <si>
     <t>EMA: Government invests in cleaning up contaminated Crown land: Media release 23 September 2026</t>
@@ -226,7 +226,7 @@
     <t>DOC has confirmed toxoplasmosis was the cause of death of a pregnant Hector’s dolphin found at Invercargill’s Oreti Beach last month.</t>
   </si>
   <si>
-    <t>2026-09-29T06:19:42.918Z</t>
+    <t>2026-09-29T06:46:24.308Z</t>
   </si>
   <si>
     <t>EMA: Toxoplasmosis confirmed as cause of death of pregnant Hector’s dolphin: Media release 22 September 2026</t>
@@ -247,7 +247,7 @@
     <t>The whitebait fishing season is open. Find out when, where and how to fish for whitebait in New Zealand and the Chatham Islands.</t>
   </si>
   <si>
-    <t>2026-09-29T06:19:09.443Z</t>
+    <t>2026-09-29T06:45:51.164Z</t>
   </si>
   <si>
     <t>EMA: Whitebaiting: Things to do</t>
@@ -271,7 +271,7 @@
     <t>Discover some of our best short walks. They’re easy to get to and great for families – there’s something for everyone.</t>
   </si>
   <si>
-    <t>2026-09-29T06:20:27.992Z</t>
+    <t>2026-09-29T06:46:46.991Z</t>
   </si>
   <si>
     <t>EMA: Short Walks: Walking and tramping</t>

</xml_diff>